<commit_message>
n8n board refresh 2026-06-05T17:40:06Z
</commit_message>
<xml_diff>
--- a/app/reports/SPCX_research.xlsx
+++ b/app/reports/SPCX_research.xlsx
@@ -615,7 +615,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-06-04 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-06-05 17:37 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>0.04470999717712403</v>
+        <v>0.04532000064849853</v>
       </c>
     </row>
     <row r="6">

</xml_diff>